<commit_message>
fix TTE, fix plot labels, and describe censoring within 1 year
</commit_message>
<xml_diff>
--- a/manuscript/tables/e-table-1-tte.xlsx
+++ b/manuscript/tables/e-table-1-tte.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gwenaubrac/Desktop/Gwen's Documents/Work/Boston University GRA/Projects/GLP1s for AD/03_analysis/repository/newer-glp1-dementia-repkit/manuscript/tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gwenaubrac/Desktop/Gwen's Documents/Work/Boston University GRA/Projects/GLP1s for AD/03_analysis/newer-glp1-dementia-repkit/manuscript/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E55314-3DF0-FE40-8F8B-54451CE54B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D2FBC1-4A73-6F42-A4E7-2E357F69BCCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19720" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
   </bookViews>
   <sheets>
     <sheet name="Target Trial Emulation" sheetId="2" r:id="rId1"/>
@@ -59,82 +59,81 @@
     <t>Treatment strategies</t>
   </si>
   <si>
-    <t xml:space="preserve">For GLP-1 agonist vs SGLT2 inhibitors trial: 
+    <t xml:space="preserve">Same as for the target trial. The date of medication initiation was defined as the date of first fill for the medication. </t>
+  </si>
+  <si>
+    <t>Treatment assignment</t>
+  </si>
+  <si>
+    <t>Outcomes</t>
+  </si>
+  <si>
+    <t>All-cause dementia diagnosis</t>
+  </si>
+  <si>
+    <t>Causal contrast of interest</t>
+  </si>
+  <si>
+    <t>Follow-up</t>
+  </si>
+  <si>
+    <t>Statistical analysis</t>
+  </si>
+  <si>
+    <t>Eligible individuals are randomly assigned to a treatment strategy at baseline (time 0).</t>
+  </si>
+  <si>
+    <t>• Kaplan-Meier estimator to obtain cumulative incidences for each treatment strategy over 2 years of follow-up
+• Cox proportional hazards model to compare the instantaneous risk of the outcome over follow-up for each treatment strategy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Follow-up starts on the day of treatment assignment and ends at occurrence of the outcome, death, loss to follow-up, end of the study (December 31st, 2025) or 2 years after baseline, whichever occurs first. Time of randomization and time of treatment initiation are aligned (time 0). </t>
+  </si>
+  <si>
+    <t>• Observational analog to intention-to-treat
+• Sensitivity analysis for observational analog to per-protocol, where individuals are censored when they discontinue or switch medications (using a 90 day grace period)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intention-to-treat
+</t>
+  </si>
+  <si>
+    <t>• Same as for the target trial. We also require at least 12 months of continuous insurance coverage prior to the index date and 90 days of continuous coverage after the index date and no prior mild cognitive impairment or neuroimaging during the 12-month baseline period. 
+• Sensitivity analysis requiring at least 6 months of continuous insurance coverage (instead of 12 months)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For GLP-1 RA vs SGLT2 inhibitors trial: 
 • Initiate use of semaglutide or tirzepatide
 • Initiate use of SGLT2 inhibitors
-For  GLP-1 agonists vs DPP4 inhibitors trial: 
+For  GLP-1 RAs vs DPP4 inhibitors trial: 
 • Initiate use of semaglutide or tirzepatide
 • Initiate use of DPP4 inhibitors
-For GLP-1 agonists vs sulfonylureas:
+For GLP-1 RAs vs sulfonylureas:
 • Initiate use of semaglutide or tirzepatide
 • Initiate use of sulfonylureas
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Same as for the target trial. The date of medication initiation was defined as the date of first fill for the medication. </t>
-  </si>
-  <si>
-    <t>Treatment assignment</t>
-  </si>
-  <si>
-    <t>Outcomes</t>
-  </si>
-  <si>
-    <t>All-cause dementia diagnosis</t>
-  </si>
-  <si>
-    <t>Causal contrast of interest</t>
-  </si>
-  <si>
-    <t>Follow-up</t>
-  </si>
-  <si>
-    <t>Statistical analysis</t>
-  </si>
-  <si>
-    <t>Eligible individuals are randomly assigned to a treatment strategy at baseline (time 0).</t>
-  </si>
-  <si>
-    <t>• Kaplan-Meier estimator to obtain cumulative incidences for each treatment strategy over 2 years of follow-up
-• Cox proportional hazards model to compare the instantaneous risk of the outcome over follow-up for each treatment strategy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Follow-up starts on the day of treatment assignment and ends at occurrence of the outcome, death, loss to follow-up, end of the study (December 31st, 2025) or 2 years after baseline, whichever occurs first. Time of randomization and time of treatment initiation are aligned (time 0). </t>
-  </si>
-  <si>
-    <t>• Follow-up starts 90 days after treatment assignment to avoid reverse causality and reduce the influence of early events. Follow-is censored at occurrence of the outcome, death, loss to follow-up, end of the study (December 31st, 2025) or 2 years after baseline, whichever occurs first. Individuals who experience an event or are censored within those first 90 days are excluded from the analysis.
-• Sensitivity analyses: 1) requiring an additional 90 days of follow-up after the initial 90 days window; 2) including individuals censored within 90 days and early events.</t>
-  </si>
-  <si>
-    <t>• Observational analog to intention-to-treat
-• Sensitivity analysis for observational analog to per-protocol, where individuals are censored when they discontinue or switch medications (using a 90 day grace period)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intention-to-treat
-</t>
+    <t xml:space="preserve">• Eligible individuals are assigned to the treatment strategy that their first medication fill is compatible with (index date). Overlap weighting based on baseline covariates are used to mimic the exchangeability one would obtain from randomization.
+• Sensitivity analyses using IPTW and entropy balancing weights instead of overlap weighting. </t>
+  </si>
+  <si>
+    <t>• Overlap-weighted Kaplan-Meier estimator to obtain cumulative incidences of each streategy over 2 years of follow-up after adjusting for baseline confounders
+• Overlap-weights Cox proportional hazards models with robust variance estimators to compare the instantaneous risk of the outcome over follow-up for each strategy after adjusting for baseline confounders
+• Additional sensitivity analysis restricting to individuals with prior use of metformin</t>
+  </si>
+  <si>
+    <t>• Follow-up starts 90 days after treatment assignment to avoid reverse causality and reduce the influence of early events. Follow-up is censored at occurrence of the outcome, death, loss to follow-up, end of the study (December 31st, 2025) or 2 years after baseline, whichever occurs first. Individuals who experience an event or are censored within those first 90 days are excluded from the analysis.
+• Sensitivity analyses: 1) starting follow-up after 6 months and excluding patients who experience the outcome during those 6 months (i.e. stricter exclusion of early events); 2) starting follow-up at index date (i.e. include early events).</t>
   </si>
   <si>
     <t>• Diagnosis of T2D
 • Age ≥60 years
 • No type 1 diabetes
 • No prior diagnosis for dementia
-• Diagnosis for overweight/obesity
 • BMI indicating overweight/obesity
 • No contra-indication for treatment (pancreatitis, thyroid cancer, gastroparesis)
-• No prior use of GLP-1 agonists (semaglutide, tirzepatide, liraglutide, dulaglutide, ablaglutide, exenative, or lixisenatide), SLGT2 inhibitors, DPP4 inhibitors, or sulfonylureas within 12 months</t>
-  </si>
-  <si>
-    <t>• Same as for the target trial. We also require at least 12 months of continuous insurance coverage prior to the index date and 90 days of continuous coverage after the index date and no prior mild cognitive impairment or neuroimaging during the 12-month baseline period. 
-• Sensitivity analysis requiring at least 6 months of continuous insurance coverage (instead of 12 months)</t>
-  </si>
-  <si>
-    <t>• Eligible individuals are assigned to the treatment strategy that their first medication fill is compatible with (index date). Overlap weighting (OW) based on baseline covariates are used to mimic the exchangeability one would obtain from randomization.
-• Sensitivity analyses using IPTW and entropy balancing weights instead of OW</t>
-  </si>
-  <si>
-    <t>• OW-weighted Kaplan-Meier estimator to obtain cumulative incidences of each streategy over 2 years of follow-up after adjusting for baseline confounders
-• OW-weights Cox proportional hazards models with robust variance estimators to compare the instantaneous risk of the outcome over follow-up for each strategy after adjusting for baseline confounders
-• Additional sensitivity analysis restricting to individuals with prior use of metformin</t>
+• No prior use of GLP-1 RAs (semaglutide, tirzepatide, liraglutide, dulaglutide, albiglutide, exenative, or lixisenatide), SLGT2 inhibitors, DPP4 inhibitors, or sulfonylureas within 12 months</t>
   </si>
 </sst>
 </file>
@@ -656,15 +655,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="255" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="238" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="259" customHeight="1" x14ac:dyDescent="0.2">
@@ -672,29 +671,29 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="168" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>4</v>
@@ -702,35 +701,35 @@
     </row>
     <row r="6" spans="1:3" ht="244" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="102" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="182" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="205" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add covariates, add aalen-johansen, add control outcomes, exclude neuro exam and cholinesterase inhibitor use
</commit_message>
<xml_diff>
--- a/manuscript/tables/e-table-1-tte.xlsx
+++ b/manuscript/tables/e-table-1-tte.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gwenaubrac/Desktop/Gwen's Documents/Work/Boston University GRA/Projects/GLP1s for AD/03_analysis/newer-glp1-dementia-repkit/manuscript/tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D2FBC1-4A73-6F42-A4E7-2E357F69BCCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E449558B-2155-4A46-BC46-45C93A9DB3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{609CF3B9-5A65-3C45-8EA5-C785028ABE13}"/>
   </bookViews>
   <sheets>
     <sheet name="Target Trial Emulation" sheetId="2" r:id="rId1"/>
@@ -98,10 +98,6 @@
 </t>
   </si>
   <si>
-    <t>• Same as for the target trial. We also require at least 12 months of continuous insurance coverage prior to the index date and 90 days of continuous coverage after the index date and no prior mild cognitive impairment or neuroimaging during the 12-month baseline period. 
-• Sensitivity analysis requiring at least 6 months of continuous insurance coverage (instead of 12 months)</t>
-  </si>
-  <si>
     <t xml:space="preserve">For GLP-1 RA vs SGLT2 inhibitors trial: 
 • Initiate use of semaglutide or tirzepatide
 • Initiate use of SGLT2 inhibitors
@@ -134,6 +130,10 @@
 • BMI indicating overweight/obesity
 • No contra-indication for treatment (pancreatitis, thyroid cancer, gastroparesis)
 • No prior use of GLP-1 RAs (semaglutide, tirzepatide, liraglutide, dulaglutide, albiglutide, exenative, or lixisenatide), SLGT2 inhibitors, DPP4 inhibitors, or sulfonylureas within 12 months</t>
+  </si>
+  <si>
+    <t>• Same as for the target trial. We also require at least 12 months of continuous insurance coverage prior to the index date and 90 days of continuous coverage after the index date and no prior mild cognitive impairment, neuroimaging, cognitive testing, or use of cholinesterase inhibitors during the 12-month baseline period. 
+• Sensitivity analysis requiring at least 6 months of continuous insurance coverage (instead of 12 months)</t>
   </si>
 </sst>
 </file>
@@ -660,10 +660,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="259" customHeight="1" x14ac:dyDescent="0.2">
@@ -671,7 +671,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>6</v>
@@ -685,7 +685,7 @@
         <v>13</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
@@ -707,7 +707,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="102" x14ac:dyDescent="0.2">
@@ -729,7 +729,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>